<commit_message>
Manual commit of automatically generated files.
Signed-off-by: Klas Magnusson <klasmagnus@gmail.com>
</commit_message>
<xml_diff>
--- a/Översikt MÖRBYLÅNGA.xlsx
+++ b/Översikt MÖRBYLÅNGA.xlsx
@@ -569,7 +569,7 @@
         <v>45177</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
         <v>44172</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
         <v>43434</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         <v>43725</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
         <v>45254</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>44245</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
         <v>43493</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
         <v>44262</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         <v>44728</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
         <v>44811</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1520,7 +1520,7 @@
         <v>45097</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
         <v>43760</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         <v>44508</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1792,7 +1792,7 @@
         <v>44155</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
         <v>45170</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1968,7 +1968,7 @@
         <v>43880</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         <v>44140</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2142,7 +2142,7 @@
         <v>44222</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         <v>44467</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         <v>45062</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2400,7 +2400,7 @@
         <v>45169</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>45267</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2572,7 +2572,7 @@
         <v>43367</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2662,7 +2662,7 @@
         <v>43446</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         <v>43493</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2832,7 +2832,7 @@
         <v>43509</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2917,7 +2917,7 @@
         <v>43690</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         <v>43725</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -3087,7 +3087,7 @@
         <v>43956</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>44077</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
         <v>44460</v>
       </c>
       <c r="C32" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
         <v>44470</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -3427,7 +3427,7 @@
         <v>45049</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -3512,7 +3512,7 @@
         <v>45084</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -3597,7 +3597,7 @@
         <v>45084</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3682,7 +3682,7 @@
         <v>45084</v>
       </c>
       <c r="C37" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
         <v>43493</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v>43496</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3881,7 +3881,7 @@
         <v>43509</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3938,7 +3938,7 @@
         <v>43509</v>
       </c>
       <c r="C41" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3995,7 +3995,7 @@
         <v>43602</v>
       </c>
       <c r="C42" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -4052,7 +4052,7 @@
         <v>43612</v>
       </c>
       <c r="C43" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
         <v>43644</v>
       </c>
       <c r="C44" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -4166,7 +4166,7 @@
         <v>43725</v>
       </c>
       <c r="C45" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         <v>43725</v>
       </c>
       <c r="C46" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -4280,7 +4280,7 @@
         <v>43749</v>
       </c>
       <c r="C47" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -4337,7 +4337,7 @@
         <v>43801</v>
       </c>
       <c r="C48" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
         <v>44026</v>
       </c>
       <c r="C49" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -4451,7 +4451,7 @@
         <v>44155</v>
       </c>
       <c r="C50" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -4508,7 +4508,7 @@
         <v>44369</v>
       </c>
       <c r="C51" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -4565,7 +4565,7 @@
         <v>44467</v>
       </c>
       <c r="C52" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -4622,7 +4622,7 @@
         <v>44544</v>
       </c>
       <c r="C53" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -4679,7 +4679,7 @@
         <v>44614</v>
       </c>
       <c r="C54" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -4741,7 +4741,7 @@
         <v>44740</v>
       </c>
       <c r="C55" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
         <v>45005</v>
       </c>
       <c r="C56" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -4855,7 +4855,7 @@
         <v>45062</v>
       </c>
       <c r="C57" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -4912,7 +4912,7 @@
         <v>45275</v>
       </c>
       <c r="C58" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4969,7 +4969,7 @@
         <v>45323</v>
       </c>
       <c r="C59" s="1" t="n">
-        <v>45337</v>
+        <v>45340</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>

</xml_diff>